<commit_message>
Put AI persona columns before human columns in Table 3.
</commit_message>
<xml_diff>
--- a/output/tables/Table3_Warning_Topic_PME_by_Sample.xlsx
+++ b/output/tables/Table3_Warning_Topic_PME_by_Sample.xlsx
@@ -15,15 +15,15 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="82" uniqueCount="63">
   <si>
-    <t>Table 3. Perceived message effectiveness by warning topic and sample, n=1,012 human participants and n=1,000 AI personas</t>
+    <t>Table 3. Perceived message effectiveness by warning topic and sample, n=1,000 AI personas and n=1,012 human participants</t>
+  </si>
+  <si>
+    <t>AI personas</t>
   </si>
   <si>
     <t>Human participants</t>
   </si>
   <si>
-    <t>AI personas</t>
-  </si>
-  <si>
     <t>Topic</t>
   </si>
   <si>
@@ -45,46 +45,52 @@
     <t>Control</t>
   </si>
   <si>
+    <t>1.82 (0.01)</t>
+  </si>
+  <si>
     <t>2.42 (0.05)</t>
   </si>
   <si>
-    <t>1.82 (0.01)</t>
-  </si>
-  <si>
     <t>[Referent]</t>
   </si>
   <si>
     <t>Addiction</t>
   </si>
   <si>
+    <t>3.12 (0.02)</t>
+  </si>
+  <si>
     <t>2.73 (0.04)</t>
   </si>
   <si>
-    <t>3.12 (0.02)</t>
+    <t>1.29 (1.25, 1.34)</t>
+  </si>
+  <si>
+    <t>&lt;0.001</t>
+  </si>
+  <si>
+    <t>2.93</t>
   </si>
   <si>
     <t>0.31 (0.22, 0.40)</t>
   </si>
   <si>
-    <t>&lt;0.001</t>
-  </si>
-  <si>
     <t>0.22</t>
   </si>
   <si>
-    <t>1.29 (1.25, 1.34)</t>
-  </si>
-  <si>
-    <t>2.93</t>
-  </si>
-  <si>
     <t>Screen time break warning</t>
   </si>
   <si>
+    <t>2.44 (0.02)</t>
+  </si>
+  <si>
     <t>2.74 (0.04)</t>
   </si>
   <si>
-    <t>2.44 (0.02)</t>
+    <t>0.62 (0.57, 0.67)</t>
+  </si>
+  <si>
+    <t>0.86</t>
   </si>
   <si>
     <t>0.32 (0.24, 0.41)</t>
@@ -93,19 +99,19 @@
     <t>0.23</t>
   </si>
   <si>
-    <t>0.62 (0.57, 0.67)</t>
-  </si>
-  <si>
-    <t>0.86</t>
-  </si>
-  <si>
     <t>Not been proven safe</t>
   </si>
   <si>
+    <t>2.94 (0.02)</t>
+  </si>
+  <si>
     <t>2.84 (0.04)</t>
   </si>
   <si>
-    <t>2.94 (0.02)</t>
+    <t>1.12 (1.07, 1.16)</t>
+  </si>
+  <si>
+    <t>2.03</t>
   </si>
   <si>
     <t>0.42 (0.33, 0.50)</t>
@@ -114,19 +120,19 @@
     <t>0.30</t>
   </si>
   <si>
-    <t>1.12 (1.07, 1.16)</t>
-  </si>
-  <si>
-    <t>2.03</t>
-  </si>
-  <si>
     <t>Sleep disruption</t>
   </si>
   <si>
+    <t>3.11 (0.02)</t>
+  </si>
+  <si>
     <t>2.89 (0.04)</t>
   </si>
   <si>
-    <t>3.11 (0.02)</t>
+    <t>1.29 (1.25, 1.33)</t>
+  </si>
+  <si>
+    <t>2.88</t>
   </si>
   <si>
     <t>0.47 (0.38, 0.55)</t>
@@ -135,19 +141,19 @@
     <t>0.34</t>
   </si>
   <si>
-    <t>1.29 (1.25, 1.33)</t>
-  </si>
-  <si>
-    <t>2.88</t>
-  </si>
-  <si>
     <t>Negative body image</t>
   </si>
   <si>
+    <t>2.93 (0.02)</t>
+  </si>
+  <si>
     <t>2.95 (0.04)</t>
   </si>
   <si>
-    <t>2.93 (0.02)</t>
+    <t>1.11 (1.07, 1.15)</t>
+  </si>
+  <si>
+    <t>1.99</t>
   </si>
   <si>
     <t>0.53 (0.44, 0.62)</t>
@@ -156,19 +162,19 @@
     <t>0.39</t>
   </si>
   <si>
-    <t>1.11 (1.07, 1.15)</t>
-  </si>
-  <si>
-    <t>1.99</t>
-  </si>
-  <si>
     <t>Depression and anxiety</t>
   </si>
   <si>
+    <t>3.24 (0.02)</t>
+  </si>
+  <si>
     <t>2.99 (0.04)</t>
   </si>
   <si>
-    <t>3.24 (0.02)</t>
+    <t>1.42 (1.38, 1.45)</t>
+  </si>
+  <si>
+    <t>4.28</t>
   </si>
   <si>
     <t>0.57 (0.47, 0.66)</t>
@@ -177,31 +183,25 @@
     <t>0.42</t>
   </si>
   <si>
-    <t>1.42 (1.38, 1.45)</t>
-  </si>
-  <si>
-    <t>4.28</t>
-  </si>
-  <si>
     <t>Mental health harms to young people</t>
   </si>
   <si>
+    <t>3.20 (0.02)</t>
+  </si>
+  <si>
     <t>3.00 (0.04)</t>
   </si>
   <si>
-    <t>3.20 (0.02)</t>
+    <t>1.38 (1.34, 1.42)</t>
+  </si>
+  <si>
+    <t>3.70</t>
   </si>
   <si>
     <t>0.58 (0.49, 0.67)</t>
   </si>
   <si>
     <t>0.43</t>
-  </si>
-  <si>
-    <t>1.38 (1.34, 1.42)</t>
-  </si>
-  <si>
-    <t>3.70</t>
   </si>
 </sst>
 </file>
@@ -637,7 +637,7 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
@@ -652,7 +652,7 @@
         <v>15</v>
       </c>
       <c r="H5">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I5" t="s">
         <v>19</v>
@@ -672,7 +672,7 @@
         <v>22</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
@@ -687,7 +687,7 @@
         <v>23</v>
       </c>
       <c r="H6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I6" t="s">
         <v>26</v>
@@ -777,7 +777,7 @@
         <v>43</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D9" t="s">
         <v>45</v>
@@ -792,7 +792,7 @@
         <v>44</v>
       </c>
       <c r="H9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I9" t="s">
         <v>47</v>
@@ -812,7 +812,7 @@
         <v>50</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="s">
         <v>52</v>
@@ -827,7 +827,7 @@
         <v>51</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10" t="s">
         <v>54</v>
@@ -847,7 +847,7 @@
         <v>57</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" t="s">
         <v>59</v>
@@ -862,7 +862,7 @@
         <v>58</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I11" t="s">
         <v>61</v>

</xml_diff>